<commit_message>
adding LA to the database
</commit_message>
<xml_diff>
--- a/Results_isofys/LeavesNumexSF2023_20251015.xlsx
+++ b/Results_isofys/LeavesNumexSF2023_20251015.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="31">
   <si>
     <t>Alchornea lojaensis</t>
   </si>
@@ -69,9 +69,6 @@
   </si>
   <si>
     <t>Myrtaceae</t>
-  </si>
-  <si>
-    <t>4966, 9683</t>
   </si>
   <si>
     <t>P</t>
@@ -791,55 +788,55 @@
         <v>7</v>
       </c>
       <c r="G1" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="H1" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="K1" s="40" t="s">
+        <v>30</v>
+      </c>
+      <c r="L1" s="41" t="s">
+        <v>29</v>
+      </c>
+      <c r="M1" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="H1" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="I1" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="J1" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="K1" s="40" t="s">
-        <v>31</v>
-      </c>
-      <c r="L1" s="41" t="s">
-        <v>30</v>
-      </c>
-      <c r="M1" s="40" t="s">
-        <v>28</v>
-      </c>
       <c r="N1" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="O1" s="33" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q1" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="O1" s="33" t="s">
-        <v>15</v>
-      </c>
-      <c r="P1" s="33" t="s">
+      <c r="R1" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="Q1" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="R1" s="33" t="s">
+      <c r="S1" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="S1" s="33" t="s">
-        <v>20</v>
-      </c>
       <c r="T1" s="33" t="s">
+        <v>20</v>
+      </c>
+      <c r="U1" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="U1" s="33" t="s">
+      <c r="V1" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="V1" s="33" t="s">
+      <c r="W1" s="33" t="s">
         <v>23</v>
-      </c>
-      <c r="W1" s="33" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -1067,8 +1064,8 @@
       <c r="D5" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="23" t="s">
-        <v>11</v>
+      <c r="E5" s="23">
+        <v>4966</v>
       </c>
       <c r="F5" s="26">
         <v>90</v>
@@ -1481,7 +1478,7 @@
         <v>2</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C11" s="35" t="s">
         <v>10</v>
@@ -1553,7 +1550,7 @@
         <v>2</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="20" t="s">
         <v>9</v>
@@ -1625,7 +1622,7 @@
         <v>2</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C13" s="20" t="s">
         <v>10</v>
@@ -1697,7 +1694,7 @@
         <v>2</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C14" s="20" t="s">
         <v>9</v>
@@ -1767,7 +1764,7 @@
         <v>2</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C15" s="35" t="s">
         <v>9</v>
@@ -1839,7 +1836,7 @@
         <v>2</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C16" s="35" t="s">
         <v>10</v>
@@ -1911,7 +1908,7 @@
         <v>2</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C17" s="35" t="s">
         <v>9</v>
@@ -1981,7 +1978,7 @@
         <v>3</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C18" s="37" t="s">
         <v>9</v>
@@ -2053,7 +2050,7 @@
         <v>3</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C19" s="37" t="s">
         <v>10</v>
@@ -2125,7 +2122,7 @@
         <v>3</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C20" s="20" t="s">
         <v>9</v>
@@ -2195,7 +2192,7 @@
         <v>3</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C21" s="35" t="s">
         <v>10</v>
@@ -2265,7 +2262,7 @@
         <v>3</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C22" s="35" t="s">
         <v>9</v>
@@ -2335,7 +2332,7 @@
         <v>3</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C23" s="35" t="s">
         <v>10</v>
@@ -2405,7 +2402,7 @@
         <v>4</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C24" s="20" t="s">
         <v>9</v>
@@ -2475,7 +2472,7 @@
         <v>4</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C25" s="38" t="s">
         <v>10</v>
@@ -2545,7 +2542,7 @@
         <v>4</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C26" s="35" t="s">
         <v>10</v>
@@ -2615,7 +2612,7 @@
         <v>4</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C27" s="20" t="s">
         <v>10</v>
@@ -2685,7 +2682,7 @@
         <v>4</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C28" s="35" t="s">
         <v>9</v>
@@ -2755,7 +2752,7 @@
         <v>4</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C29" s="37" t="s">
         <v>9</v>
@@ -2825,7 +2822,7 @@
         <v>4</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C30" s="35" t="s">
         <v>10</v>
@@ -2897,7 +2894,7 @@
         <v>4</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C31" s="27" t="s">
         <v>9</v>
@@ -2967,7 +2964,7 @@
         <v>6</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C32" s="35" t="s">
         <v>10</v>
@@ -3039,7 +3036,7 @@
         <v>6</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C33" s="35" t="s">
         <v>9</v>
@@ -3109,7 +3106,7 @@
         <v>6</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C34" s="35" t="s">
         <v>9</v>
@@ -3179,7 +3176,7 @@
         <v>6</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C35" s="35" t="s">
         <v>10</v>
@@ -3251,7 +3248,7 @@
         <v>6</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C36" s="20" t="s">
         <v>9</v>
@@ -3321,7 +3318,7 @@
         <v>6</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C37" s="35" t="s">
         <v>10</v>
@@ -3883,7 +3880,7 @@
         <v>8</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C45" s="35" t="s">
         <v>10</v>
@@ -3953,7 +3950,7 @@
         <v>8</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C46" s="35" t="s">
         <v>9</v>
@@ -4025,7 +4022,7 @@
         <v>8</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C47" s="35" t="s">
         <v>9</v>
@@ -4095,7 +4092,7 @@
         <v>8</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C48" s="20" t="s">
         <v>9</v>
@@ -4165,7 +4162,7 @@
         <v>8</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C49" s="38" t="s">
         <v>10</v>
@@ -4235,7 +4232,7 @@
         <v>9</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C50" s="35" t="s">
         <v>9</v>
@@ -4307,7 +4304,7 @@
         <v>9</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C51" s="37" t="s">
         <v>9</v>
@@ -4379,7 +4376,7 @@
         <v>11</v>
       </c>
       <c r="B52" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C52" s="20" t="s">
         <v>9</v>
@@ -4449,7 +4446,7 @@
         <v>11</v>
       </c>
       <c r="B53" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C53" s="35" t="s">
         <v>10</v>
@@ -4521,7 +4518,7 @@
         <v>11</v>
       </c>
       <c r="B54" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C54" s="20" t="s">
         <v>9</v>
@@ -4591,7 +4588,7 @@
         <v>11</v>
       </c>
       <c r="B55" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C55" s="37" t="s">
         <v>10</v>
@@ -4661,7 +4658,7 @@
         <v>11</v>
       </c>
       <c r="B56" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C56" s="20" t="s">
         <v>9</v>
@@ -4731,7 +4728,7 @@
         <v>11</v>
       </c>
       <c r="B57" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C57" s="35" t="s">
         <v>9</v>
@@ -4801,7 +4798,7 @@
         <v>11</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C58" s="37" t="s">
         <v>10</v>
@@ -5225,7 +5222,7 @@
         <v>13</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C64" s="35" t="s">
         <v>9</v>
@@ -5297,7 +5294,7 @@
         <v>13</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C65" s="35" t="s">
         <v>10</v>
@@ -5367,7 +5364,7 @@
         <v>13</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C66" s="20" t="s">
         <v>9</v>
@@ -5437,7 +5434,7 @@
         <v>13</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C67" s="35" t="s">
         <v>9</v>
@@ -5507,7 +5504,7 @@
         <v>13</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C68" s="38" t="s">
         <v>10</v>
@@ -5577,7 +5574,7 @@
         <v>14</v>
       </c>
       <c r="B69" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C69" s="35" t="s">
         <v>10</v>
@@ -5647,7 +5644,7 @@
         <v>14</v>
       </c>
       <c r="B70" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C70" s="37" t="s">
         <v>10</v>
@@ -5719,7 +5716,7 @@
         <v>14</v>
       </c>
       <c r="B71" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C71" s="20" t="s">
         <v>10</v>
@@ -5789,7 +5786,7 @@
         <v>14</v>
       </c>
       <c r="B72" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C72" s="35" t="s">
         <v>9</v>
@@ -5861,7 +5858,7 @@
         <v>14</v>
       </c>
       <c r="B73" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C73" s="37" t="s">
         <v>10</v>
@@ -5931,7 +5928,7 @@
         <v>14</v>
       </c>
       <c r="B74" s="11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C74" s="35" t="s">
         <v>10</v>
@@ -6001,7 +5998,7 @@
         <v>16</v>
       </c>
       <c r="B75" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C75" s="35" t="s">
         <v>10</v>
@@ -6071,7 +6068,7 @@
         <v>16</v>
       </c>
       <c r="B76" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C76" s="20" t="s">
         <v>10</v>
@@ -6141,7 +6138,7 @@
         <v>16</v>
       </c>
       <c r="B77" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C77" s="35" t="s">
         <v>9</v>
@@ -6211,7 +6208,7 @@
         <v>16</v>
       </c>
       <c r="B78" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C78" s="37" t="s">
         <v>9</v>
@@ -6281,7 +6278,7 @@
         <v>16</v>
       </c>
       <c r="B79" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C79" s="20" t="s">
         <v>10</v>
@@ -6351,7 +6348,7 @@
         <v>16</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C80" s="35" t="s">
         <v>10</v>
@@ -6845,7 +6842,7 @@
         <v>18</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C87" s="37" t="s">
         <v>10</v>
@@ -6917,7 +6914,7 @@
         <v>18</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C88" s="20" t="s">
         <v>10</v>
@@ -6987,7 +6984,7 @@
         <v>18</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C89" s="35" t="s">
         <v>9</v>
@@ -7059,7 +7056,7 @@
         <v>18</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C90" s="20" t="s">
         <v>10</v>
@@ -7129,7 +7126,7 @@
         <v>19</v>
       </c>
       <c r="B91" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C91" s="37" t="s">
         <v>10</v>
@@ -7201,7 +7198,7 @@
         <v>19</v>
       </c>
       <c r="B92" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C92" s="35" t="s">
         <v>9</v>
@@ -7273,7 +7270,7 @@
         <v>19</v>
       </c>
       <c r="B93" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C93" s="20" t="s">
         <v>10</v>
@@ -7343,7 +7340,7 @@
         <v>19</v>
       </c>
       <c r="B94" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C94" s="35" t="s">
         <v>10</v>

</xml_diff>